<commit_message>
Drivers: company-managed share of openings 63% (58–68%) after FY25 actuals
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016tKeYTtjF85cuvm1dpYiVi
</commit_message>
<xml_diff>
--- a/model/GRG_model_v0.3.xlsx
+++ b/model/GRG_model_v0.3.xlsx
@@ -1323,7 +1323,7 @@
     <t xml:space="preserve">%</t>
   </si>
   <si>
-    <t xml:space="preserve">Rising: 55%, 57%, 60% (FY22–FY24)</t>
+    <t xml:space="preserve">Rising: 55%, 57%, 60%, 66% (FY22–FY25); revised 11 Oct after FY25 actuals</t>
   </si>
   <si>
     <t xml:space="preserve">Company-managed like-for-like growth</t>
@@ -7027,11 +7027,11 @@
       </c>
       <c r="I15" s="28" t="n">
         <f aca="false">-I150-I151</f>
-        <v>-19.3093542349088</v>
+        <v>-19.3352119466542</v>
       </c>
       <c r="J15" s="28" t="n">
         <f aca="false">-J150-J151</f>
-        <v>-19.851134861956</v>
+        <v>-19.9040816050538</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7064,11 +7064,11 @@
       </c>
       <c r="I16" s="44" t="n">
         <f aca="false">I13+I14+I15</f>
-        <v>-29.3093542349088</v>
+        <v>-29.3352119466542</v>
       </c>
       <c r="J16" s="44" t="n">
         <f aca="false">J13+J14+J15</f>
-        <v>-24.851134861956</v>
+        <v>-24.9040816050538</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7104,11 +7104,11 @@
       </c>
       <c r="I17" s="28" t="n">
         <f aca="false">-Drivers!$D$18*I16</f>
-        <v>7.62043210107628</v>
+        <v>7.62715510613009</v>
       </c>
       <c r="J17" s="28" t="n">
         <f aca="false">-Drivers!$E$18*J16</f>
-        <v>6.46129506410856</v>
+        <v>6.47506121731399</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7141,11 +7141,11 @@
       </c>
       <c r="I18" s="44" t="n">
         <f aca="false">I16+I17</f>
-        <v>-21.6889221338325</v>
+        <v>-21.7080568405241</v>
       </c>
       <c r="J18" s="44" t="n">
         <f aca="false">J16+J17</f>
-        <v>-18.3898397978475</v>
+        <v>-18.4290203877398</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7346,11 +7346,11 @@
       </c>
       <c r="I25" s="44" t="n">
         <f aca="false">I16-I21-I22</f>
-        <v>-19.3093542349088</v>
+        <v>-19.3352119466542</v>
       </c>
       <c r="J25" s="44" t="n">
         <f aca="false">J16-J21-J22</f>
-        <v>-19.851134861956</v>
+        <v>-19.9040816050538</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7787,15 +7787,15 @@
       </c>
       <c r="H41" s="30" t="n">
         <f aca="false">G41+(1-Drivers!$C$7)*Drivers!$C$6</f>
-        <v>644</v>
+        <v>640.85</v>
       </c>
       <c r="I41" s="30" t="n">
         <f aca="false">H41+(1-Drivers!$D$7)*Drivers!$D$6</f>
-        <v>688</v>
+        <v>681.55</v>
       </c>
       <c r="J41" s="30" t="n">
         <f aca="false">I41+(1-Drivers!$E$7)*Drivers!$E$6</f>
-        <v>732</v>
+        <v>722.25</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7824,15 +7824,15 @@
       </c>
       <c r="H42" s="30" t="n">
         <f aca="false">IF(H41="","",H40-H41)</f>
-        <v>2200</v>
+        <v>2203.15</v>
       </c>
       <c r="I42" s="30" t="n">
         <f aca="false">IF(I41="","",I40-I41)</f>
-        <v>2266</v>
+        <v>2272.45</v>
       </c>
       <c r="J42" s="30" t="n">
         <f aca="false">IF(J41="","",J40-J41)</f>
-        <v>2332</v>
+        <v>2341.75</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8187,15 +8187,15 @@
       </c>
       <c r="H54" s="28" t="n">
         <f aca="false">G54*H42/G42</f>
-        <v>425.175479644361</v>
+        <v>425.784253626579</v>
       </c>
       <c r="I54" s="28" t="n">
         <f aca="false">H54*I42/H42</f>
-        <v>437.930744033692</v>
+        <v>439.177281235377</v>
       </c>
       <c r="J54" s="28" t="n">
         <f aca="false">I54*J42/I42</f>
-        <v>450.686008423023</v>
+        <v>452.570308844174</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8261,15 +8261,15 @@
       </c>
       <c r="H56" s="44" t="n">
         <f aca="false">SUM(H52:H55)</f>
-        <v>1360.20197964436</v>
+        <v>1360.81075362658</v>
       </c>
       <c r="I56" s="44" t="n">
         <f aca="false">SUM(I52:I55)</f>
-        <v>1409.49396653369</v>
+        <v>1410.74050373538</v>
       </c>
       <c r="J56" s="44" t="n">
         <f aca="false">SUM(J52:J55)</f>
-        <v>1448.66174188552</v>
+        <v>1450.54604230667</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8455,15 +8455,15 @@
       </c>
       <c r="H61" s="28" t="n">
         <f aca="false">H113</f>
-        <v>-210.095167646701</v>
+        <v>-210.040923379036</v>
       </c>
       <c r="I61" s="28" t="n">
         <f aca="false">I113</f>
-        <v>-359.882446244934</v>
+        <v>-359.790509355931</v>
       </c>
       <c r="J61" s="28" t="n">
         <f aca="false">J113</f>
-        <v>-483.794438638808</v>
+        <v>-483.684855011667</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8492,15 +8492,15 @@
       </c>
       <c r="H62" s="44" t="n">
         <f aca="false">SUM(H57:H61)</f>
-        <v>-210.095167646701</v>
+        <v>-210.040923379036</v>
       </c>
       <c r="I62" s="44" t="n">
         <f aca="false">SUM(I57:I61)</f>
-        <v>-359.882446244934</v>
+        <v>-359.790509355931</v>
       </c>
       <c r="J62" s="44" t="n">
         <f aca="false">SUM(J57:J61)</f>
-        <v>-483.794438638808</v>
+        <v>-483.684855011667</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8529,15 +8529,15 @@
       </c>
       <c r="H63" s="44" t="n">
         <f aca="false">H56+H62</f>
-        <v>1150.10681199766</v>
+        <v>1150.76983024754</v>
       </c>
       <c r="I63" s="44" t="n">
         <f aca="false">I56+I62</f>
-        <v>1049.61152028876</v>
+        <v>1050.94999437945</v>
       </c>
       <c r="J63" s="44" t="n">
         <f aca="false">J56+J62</f>
-        <v>964.867303246715</v>
+        <v>966.861187295007</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8646,15 +8646,15 @@
       </c>
       <c r="H66" s="28" t="n">
         <f aca="false">-H146*Drivers!$C$35</f>
-        <v>-64.3653907346748</v>
+        <v>-64.4575502714085</v>
       </c>
       <c r="I66" s="28" t="n">
         <f aca="false">-I146*Drivers!$D$35</f>
-        <v>-66.296352456715</v>
+        <v>-66.4850600795508</v>
       </c>
       <c r="J66" s="28" t="n">
         <f aca="false">-J146*Drivers!$E$35</f>
-        <v>-68.2273141787553</v>
+        <v>-68.512569887693</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8720,15 +8720,15 @@
       </c>
       <c r="H68" s="44" t="n">
         <f aca="false">SUM(H64:H67)</f>
-        <v>-111.765390734675</v>
+        <v>-111.857550271409</v>
       </c>
       <c r="I68" s="44" t="n">
         <f aca="false">SUM(I64:I67)</f>
-        <v>-88.696352456715</v>
+        <v>-88.8850600795508</v>
       </c>
       <c r="J68" s="44" t="n">
         <f aca="false">SUM(J64:J67)</f>
-        <v>-80.6273141787553</v>
+        <v>-80.912569887693</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8834,15 +8834,15 @@
       </c>
       <c r="H71" s="28" t="n">
         <f aca="false">-H146*(1-Drivers!$C$35)</f>
-        <v>-398.694974262985</v>
+        <v>-399.265832976135</v>
       </c>
       <c r="I71" s="28" t="n">
         <f aca="false">-I146*(1-Drivers!$D$35)</f>
-        <v>-410.655823490875</v>
+        <v>-411.824724665419</v>
       </c>
       <c r="J71" s="28" t="n">
         <f aca="false">-J146*(1-Drivers!$E$35)</f>
-        <v>-422.616672718765</v>
+        <v>-424.383616354703</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8982,15 +8982,15 @@
       </c>
       <c r="H75" s="44" t="n">
         <f aca="false">SUM(H69:H74)</f>
-        <v>-529.086889262985</v>
+        <v>-529.657747976135</v>
       </c>
       <c r="I75" s="44" t="n">
         <f aca="false">SUM(I69:I74)</f>
-        <v>-545.066777965875</v>
+        <v>-546.235679140419</v>
       </c>
       <c r="J75" s="44" t="n">
         <f aca="false">SUM(J69:J74)</f>
-        <v>-559.93300339964</v>
+        <v>-561.699947035578</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9019,15 +9019,15 @@
       </c>
       <c r="H76" s="44" t="n">
         <f aca="false">H68+H75</f>
-        <v>-640.85227999766</v>
+        <v>-641.515298247543</v>
       </c>
       <c r="I76" s="44" t="n">
         <f aca="false">I68+I75</f>
-        <v>-633.76313042259</v>
+        <v>-635.120739219969</v>
       </c>
       <c r="J76" s="44" t="n">
         <f aca="false">J68+J75</f>
-        <v>-640.560317578395</v>
+        <v>-642.612516923271</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9060,11 +9060,11 @@
       </c>
       <c r="I77" s="44" t="n">
         <f aca="false">I63+I76</f>
-        <v>415.848389866168</v>
+        <v>415.829255159476</v>
       </c>
       <c r="J77" s="44" t="n">
         <f aca="false">J63+J76</f>
-        <v>324.30698566832</v>
+        <v>324.248670371736</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9211,11 +9211,11 @@
       </c>
       <c r="I81" s="28" t="n">
         <f aca="false">H81+I18+I108</f>
-        <v>388.348389866168</v>
+        <v>388.329255159476</v>
       </c>
       <c r="J81" s="28" t="n">
         <f aca="false">I81+J18+J108</f>
-        <v>296.80698566832</v>
+        <v>296.748670371736</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9248,11 +9248,11 @@
       </c>
       <c r="I82" s="44" t="n">
         <f aca="false">SUM(I78:I81)</f>
-        <v>415.848389866168</v>
+        <v>415.829255159476</v>
       </c>
       <c r="J82" s="44" t="n">
         <f aca="false">SUM(J78:J81)</f>
-        <v>324.30698566832</v>
+        <v>324.248670371736</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9351,15 +9351,15 @@
       </c>
       <c r="H87" s="28" t="n">
         <f aca="false">H61+H69</f>
-        <v>-235.095167646701</v>
+        <v>-235.040923379036</v>
       </c>
       <c r="I87" s="28" t="n">
         <f aca="false">I61+I69</f>
-        <v>-384.882446244934</v>
+        <v>-384.790509355931</v>
       </c>
       <c r="J87" s="28" t="n">
         <f aca="false">J61+J69</f>
-        <v>-508.794438638808</v>
+        <v>-508.684855011667</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9388,15 +9388,15 @@
       </c>
       <c r="H88" s="28" t="n">
         <f aca="false">H66+H71</f>
-        <v>-463.06036499766</v>
+        <v>-463.723383247543</v>
       </c>
       <c r="I88" s="28" t="n">
         <f aca="false">I66+I71</f>
-        <v>-476.95217594759</v>
+        <v>-478.30978474497</v>
       </c>
       <c r="J88" s="28" t="n">
         <f aca="false">J66+J71</f>
-        <v>-490.84398689752</v>
+        <v>-492.896186242396</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9425,15 +9425,15 @@
       </c>
       <c r="H89" s="28" t="n">
         <f aca="false">H87+H88</f>
-        <v>-698.155532644361</v>
+        <v>-698.764306626579</v>
       </c>
       <c r="I89" s="28" t="n">
         <f aca="false">I87+I88</f>
-        <v>-861.834622192524</v>
+        <v>-863.100294100901</v>
       </c>
       <c r="J89" s="28" t="n">
         <f aca="false">J87+J88</f>
-        <v>-999.638425536328</v>
+        <v>-1001.58104125406</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9480,11 +9480,11 @@
       </c>
       <c r="I92" s="28" t="n">
         <f aca="false">I13+I145+I144+I147-(I57-H57)-(I58-H58)-(I64-H64)-(I67-H67)</f>
-        <v>165.743109039541</v>
+        <v>165.846600616519</v>
       </c>
       <c r="J92" s="28" t="n">
         <f aca="false">J13+J145+J144+J147-(J57-I57)-(J58-I58)-(J64-I64)-(J67-I67)</f>
-        <v>193.035715523228</v>
+        <v>193.247626847514</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9517,11 +9517,11 @@
       </c>
       <c r="I93" s="28" t="n">
         <f aca="false">I17-(I72-H72)</f>
-        <v>11.6394715760763</v>
+        <v>11.6461945811301</v>
       </c>
       <c r="J93" s="28" t="n">
         <f aca="false">J17-(J72-I72)</f>
-        <v>9.36667126998357</v>
+        <v>9.38043742318899</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9591,11 +9591,11 @@
       </c>
       <c r="I95" s="28" t="n">
         <f aca="false">-I150</f>
-        <v>-18.0593542349088</v>
+        <v>-18.0852119466542</v>
       </c>
       <c r="J95" s="28" t="n">
         <f aca="false">-J150</f>
-        <v>-18.601134861956</v>
+        <v>-18.6540816050538</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9668,11 +9668,11 @@
       </c>
       <c r="I97" s="44" t="n">
         <f aca="false">SUM(I92:I96)</f>
-        <v>158.073226380709</v>
+        <v>158.157583250994</v>
       </c>
       <c r="J97" s="44" t="n">
         <f aca="false">SUM(J92:J96)</f>
-        <v>182.551251931255</v>
+        <v>182.723982665649</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10111,15 +10111,15 @@
       </c>
       <c r="H109" s="28" t="n">
         <f aca="false">-H149</f>
-        <v>-69.125114646701</v>
+        <v>-69.070870379036</v>
       </c>
       <c r="I109" s="28" t="n">
         <f aca="false">-I149</f>
-        <v>-71.1432849789424</v>
+        <v>-71.1899492278895</v>
       </c>
       <c r="J109" s="28" t="n">
         <f aca="false">-J149</f>
-        <v>-73.3116799251287</v>
+        <v>-73.4667639213851</v>
       </c>
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10148,15 +10148,15 @@
       </c>
       <c r="H110" s="44" t="n">
         <f aca="false">SUM(H103:H109)</f>
-        <v>-139.436114646701</v>
+        <v>-139.381870379036</v>
       </c>
       <c r="I110" s="44" t="n">
         <f aca="false">SUM(I103:I109)</f>
-        <v>-142.860504978942</v>
+        <v>-142.907169227889</v>
       </c>
       <c r="J110" s="44" t="n">
         <f aca="false">SUM(J103:J109)</f>
-        <v>-146.463244325129</v>
+        <v>-146.618328321385</v>
       </c>
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10185,15 +10185,15 @@
       </c>
       <c r="H111" s="44" t="n">
         <f aca="false">H97+H102+H110</f>
-        <v>-280.895167646701</v>
+        <v>-280.840923379036</v>
       </c>
       <c r="I111" s="44" t="n">
         <f aca="false">I97+I102+I110</f>
-        <v>-149.787278598233</v>
+        <v>-149.749585976895</v>
       </c>
       <c r="J111" s="44" t="n">
         <f aca="false">J97+J102+J110</f>
-        <v>-123.911992393873</v>
+        <v>-123.894345655736</v>
       </c>
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10226,11 +10226,11 @@
       </c>
       <c r="I112" s="28" t="n">
         <f aca="false">H113</f>
-        <v>-210.095167646701</v>
+        <v>-210.040923379036</v>
       </c>
       <c r="J112" s="28" t="n">
         <f aca="false">I113</f>
-        <v>-359.882446244934</v>
+        <v>-359.790509355931</v>
       </c>
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10259,15 +10259,15 @@
       </c>
       <c r="H113" s="44" t="n">
         <f aca="false">H112+H111</f>
-        <v>-210.095167646701</v>
+        <v>-210.040923379036</v>
       </c>
       <c r="I113" s="44" t="n">
         <f aca="false">I112+I111</f>
-        <v>-359.882446244934</v>
+        <v>-359.790509355931</v>
       </c>
       <c r="J113" s="44" t="n">
         <f aca="false">J112+J111</f>
-        <v>-483.794438638808</v>
+        <v>-483.684855011667</v>
       </c>
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10375,15 +10375,15 @@
       </c>
       <c r="H118" s="28" t="n">
         <f aca="false">H97+H117+H109</f>
-        <v>-210.584167646701</v>
+        <v>-210.529923379036</v>
       </c>
       <c r="I118" s="28" t="n">
         <f aca="false">I97+I117+I109</f>
-        <v>-78.0700585982335</v>
+        <v>-78.0323659768951</v>
       </c>
       <c r="J118" s="28" t="n">
         <f aca="false">J97+J117+J109</f>
-        <v>-50.7604279938735</v>
+        <v>-50.7427812557359</v>
       </c>
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11041,15 +11041,15 @@
       </c>
       <c r="H146" s="28" t="n">
         <f aca="false">-(G66+G71)*H42/G42</f>
-        <v>463.06036499766</v>
+        <v>463.723383247543</v>
       </c>
       <c r="I146" s="28" t="n">
         <f aca="false">-(H66+H71)*I42/H42</f>
-        <v>476.95217594759</v>
+        <v>478.30978474497</v>
       </c>
       <c r="J146" s="28" t="n">
         <f aca="false">-(I66+I71)*J42/I42</f>
-        <v>490.84398689752</v>
+        <v>492.896186242396</v>
       </c>
     </row>
     <row r="147" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11062,11 +11062,11 @@
       </c>
       <c r="I147" s="28" t="n">
         <f aca="false">H54*Drivers!$D$29</f>
-        <v>72.2798315395414</v>
+        <v>72.3833231165185</v>
       </c>
       <c r="J147" s="28" t="n">
         <f aca="false">I54*Drivers!$E$29</f>
-        <v>74.4482264857277</v>
+        <v>74.660137810014</v>
       </c>
     </row>
     <row r="148" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11078,15 +11078,15 @@
       </c>
       <c r="H148" s="28" t="n">
         <f aca="false">H54-G54+H147</f>
-        <v>82.3854796443613</v>
+        <v>82.9942536265794</v>
       </c>
       <c r="I148" s="28" t="n">
         <f aca="false">I54-H54+I147</f>
-        <v>85.0350959288722</v>
+        <v>85.7763507253158</v>
       </c>
       <c r="J148" s="28" t="n">
         <f aca="false">J54-I54+J147</f>
-        <v>87.2034908750585</v>
+        <v>88.0531654188115</v>
       </c>
     </row>
     <row r="149" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11098,15 +11098,15 @@
       </c>
       <c r="H149" s="28" t="n">
         <f aca="false">-(G66+G71)+H148-H146</f>
-        <v>69.125114646701</v>
+        <v>69.070870379036</v>
       </c>
       <c r="I149" s="28" t="n">
         <f aca="false">-(H66+H71)+I148-I146</f>
-        <v>71.1432849789424</v>
+        <v>71.1899492278895</v>
       </c>
       <c r="J149" s="28" t="n">
         <f aca="false">-(I66+I71)+J148-J146</f>
-        <v>73.3116799251287</v>
+        <v>73.4667639213851</v>
       </c>
     </row>
     <row r="150" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11119,11 +11119,11 @@
       </c>
       <c r="I150" s="28" t="n">
         <f aca="false">-(H66+H71)*Drivers!$D$30</f>
-        <v>18.0593542349088</v>
+        <v>18.0852119466542</v>
       </c>
       <c r="J150" s="28" t="n">
         <f aca="false">-(I66+I71)*Drivers!$E$30</f>
-        <v>18.601134861956</v>
+        <v>18.6540816050538</v>
       </c>
     </row>
     <row r="151" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11408,31 +11408,31 @@
         <v>335</v>
       </c>
       <c r="C7" s="31" t="n">
-        <v>0.6</v>
+        <v>0.63</v>
       </c>
       <c r="D7" s="31" t="n">
-        <v>0.6</v>
+        <v>0.63</v>
       </c>
       <c r="E7" s="31" t="n">
-        <v>0.6</v>
+        <v>0.63</v>
       </c>
       <c r="F7" s="31" t="n">
-        <v>0.55</v>
+        <v>0.58</v>
       </c>
       <c r="G7" s="31" t="n">
-        <v>0.65</v>
+        <v>0.68</v>
       </c>
       <c r="H7" s="31" t="n">
-        <v>0.55</v>
+        <v>0.58</v>
       </c>
       <c r="I7" s="31" t="n">
-        <v>0.65</v>
+        <v>0.68</v>
       </c>
       <c r="J7" s="31" t="n">
-        <v>0.55</v>
+        <v>0.58</v>
       </c>
       <c r="K7" s="31" t="n">
-        <v>0.65</v>
+        <v>0.68</v>
       </c>
       <c r="L7" s="16" t="s">
         <v>336</v>

</xml_diff>